<commit_message>
Restore 33 files clobbered by a stale cross-machine sync
Commit a457e48 unintentionally swept stale versions synced from the
other machine (whose git state shares this repo via OneDrive): both
bank qmds, the rebuilt sample test and workbook, nine answer workbooks,
the bushels fix, sidebar links, and more. All restored from a457e48^;
module03b comes from the newer OneDrive conflict copy; the orphaned
q040.xlsx is re-removed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q02.xlsx
+++ b/practice/answers/s1_q02.xlsx
@@ -1,66 +1,158 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr/>
-  <workbookProtection/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_884D9827905596AFE448FC555F7B8E3B851EEC8A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05A1834C-98D6-4321-A312-8190AAD250A5}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Answer" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Canola</t>
+  </si>
+  <si>
+    <t>Wheat</t>
+  </si>
+  <si>
+    <t>Barley</t>
+  </si>
+  <si>
+    <t>Rev Canola ($/ac)</t>
+  </si>
+  <si>
+    <t>Rev Wheat ($/ac)</t>
+  </si>
+  <si>
+    <t>Rev Barley ($/ac)</t>
+  </si>
+  <si>
+    <t>North</t>
+  </si>
+  <si>
+    <t>South</t>
+  </si>
+  <si>
+    <t>Creek</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Rented</t>
+  </si>
+  <si>
+    <t>Price ($/bu)</t>
+  </si>
+  <si>
+    <t>Average (d):</t>
+  </si>
+  <si>
+    <t>(b) Top-left formula: =B2*B$8. The row of the price reference is locked (the 8), so filling down keeps pointing at the price row; the column is left free, so filling across moves from the canola price to the wheat and barley prices.</t>
+  </si>
+  <si>
+    <t>(c) With a fully absolute reference like $B$8, every copy of the formula would multiply by the canola price -- the wheat and barley revenue columns would silently be wrong, and Excel would show no error.</t>
+  </si>
+  <si>
+    <t>(e) Canola earns the highest average revenue per acre, about $570/ac -- roughly $143/ac more than wheat (about $427/ac), with barley third (about $348/ac).</t>
+  </si>
+  <si>
+    <t>Legend: colours mark question parts</t>
+  </si>
+  <si>
+    <t>Part (a)</t>
+  </si>
+  <si>
+    <t>Part (b)</t>
+  </si>
+  <si>
+    <t>Part (c)</t>
+  </si>
+  <si>
+    <t>Part (d)</t>
+  </si>
+  <si>
+    <t>Part (e)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFE2F3"/>
+        <fgColor rgb="FFCFE2F3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
+        <fgColor rgb="FFD9D2E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,98 +168,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -455,296 +489,257 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="4" width="9" customWidth="1"/>
+    <col min="6" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Canola</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Wheat</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Barley</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Rev Canola ($/ac)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Rev Wheat ($/ac)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Rev Barley ($/ac)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>North</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>41.2</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>52.4</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>63.1</v>
       </c>
       <c r="F2" s="2">
         <f>B2*B$8</f>
-        <v/>
+        <v>585.04</v>
       </c>
       <c r="G2" s="2">
         <f>C2*C$8</f>
-        <v/>
+        <v>437.53999999999996</v>
       </c>
       <c r="H2" s="2">
         <f>D2*D$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+        <v>353.36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>38.6</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>49.8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>58.7</v>
       </c>
       <c r="F3" s="2">
         <f>B3*B$8</f>
-        <v/>
+        <v>548.12</v>
       </c>
       <c r="G3" s="2">
         <f>C3*C$8</f>
-        <v/>
+        <v>415.83</v>
       </c>
       <c r="H3" s="2">
         <f>D3*D$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Creek</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+        <v>328.71999999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>44.8</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>55.2</v>
       </c>
-      <c r="D4" t="n">
-        <v>66.40000000000001</v>
+      <c r="D4">
+        <v>66.400000000000006</v>
       </c>
       <c r="F4" s="2">
         <f>B4*B$8</f>
-        <v/>
+        <v>636.16</v>
       </c>
       <c r="G4" s="2">
         <f>C4*C$8</f>
-        <v/>
+        <v>460.92</v>
       </c>
       <c r="H4" s="2">
         <f>D4*D$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+        <v>371.84000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>36.1</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>47.3</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>61.9</v>
       </c>
       <c r="F5" s="2">
         <f>B5*B$8</f>
-        <v/>
+        <v>512.62</v>
       </c>
       <c r="G5" s="2">
         <f>C5*C$8</f>
-        <v/>
+        <v>394.95499999999998</v>
       </c>
       <c r="H5" s="2">
         <f>D5*D$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Rented</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+        <v>346.64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>39.9</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>51</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>60.2</v>
       </c>
       <c r="F6" s="2">
         <f>B6*B$8</f>
-        <v/>
+        <v>566.57999999999993</v>
       </c>
       <c r="G6" s="2">
         <f>C6*C$8</f>
-        <v/>
+        <v>425.84999999999997</v>
       </c>
       <c r="H6" s="2">
         <f>D6*D$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Price ($/bu)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+        <v>337.12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
         <v>14.2</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>8.35</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>5.6</v>
       </c>
     </row>
-    <row r="9">
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>Average (d):</t>
-        </is>
+    <row r="9" spans="1:8">
+      <c r="E9" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F9" s="3">
         <f>AVERAGE(F2:F6)</f>
-        <v/>
+        <v>569.70399999999995</v>
       </c>
       <c r="G9" s="3">
         <f>AVERAGE(G2:G6)</f>
-        <v/>
+        <v>427.01899999999995</v>
       </c>
       <c r="H9" s="3">
         <f>AVERAGE(H2:H6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="64" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>(b) Top-left formula: =B2*B$8. The row of the price reference is locked (the 8), so filling down keeps pointing at the price row; the column is left free, so filling across moves from the canola price to the wheat and barley prices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="64" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>(c) With a fully absolute reference like $B$8, every copy of the formula would multiply by the canola price -- the wheat and barley revenue columns would silently be wrong, and Excel would show no error.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>(e) Canola earns the highest average revenue per acre, about $570/ac -- roughly $143/ac more than wheat (about $427/ac), with barley third (about $348/ac).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Legend: colours mark question parts</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Part (a)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Part (b)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>Part (c)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>Part (d)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Part (e)</t>
-        </is>
+        <v>347.53599999999994</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="63.95" customHeight="1">
+      <c r="A11" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+    </row>
+    <row r="12" spans="1:8" ht="63.95" customHeight="1">
+      <c r="A12" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" ht="63.95" customHeight="1">
+      <c r="A13" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="8" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>